<commit_message>
walk through the design and nine contrasts once for every grouping
</commit_message>
<xml_diff>
--- a/03_Group_comparisons/HRvLR/01_Design_Contrasts/c_data/design_contrasts.xlsx
+++ b/03_Group_comparisons/HRvLR/01_Design_Contrasts/c_data/design_contrasts.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="201">
   <si>
     <t>sheet</t>
   </si>
@@ -318,12 +318,24 @@
     <t>1.2.1</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
   </si>
   <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
     <t>foreach</t>
   </si>
   <si>
@@ -375,6 +387,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -387,12 +411,21 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>limma</t>
   </si>
   <si>
@@ -417,6 +450,12 @@
     <t>1.5.0</t>
   </si>
   <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
     <t>pillar</t>
   </si>
   <si>
@@ -480,6 +519,12 @@
     <t>CRAN (R 4.6.1)</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -549,6 +594,12 @@
     <t>0.5.0</t>
   </si>
   <si>
+    <t>utf8</t>
+  </si>
+  <si>
+    <t>1.2.6</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
@@ -559,6 +610,12 @@
   </si>
   <si>
     <t>1.7.1</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
   </si>
   <si>
     <t>yaml</t>
@@ -1296,7 +1353,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1546,7 +1603,7 @@
         <v>109</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C23" t="s">
         <v>70</v>
@@ -1554,10 +1611,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B24" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C24" t="s">
         <v>70</v>
@@ -1565,10 +1622,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B25" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C25" t="s">
         <v>70</v>
@@ -1604,7 +1661,7 @@
         <v>119</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1637,7 +1694,7 @@
         <v>125</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1689,7 +1746,7 @@
         <v>134</v>
       </c>
       <c r="B36" t="s">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="C36" t="s">
         <v>70</v>
@@ -1697,32 +1754,32 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
+        <v>135</v>
+      </c>
+      <c r="B37" t="s">
         <v>136</v>
       </c>
-      <c r="B37" t="s">
-        <v>137</v>
-      </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
+        <v>137</v>
+      </c>
+      <c r="B38" t="s">
         <v>138</v>
       </c>
-      <c r="B38" t="s">
-        <v>139</v>
-      </c>
       <c r="C38" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>139</v>
+      </c>
+      <c r="B39" t="s">
         <v>140</v>
-      </c>
-      <c r="B39" t="s">
-        <v>141</v>
       </c>
       <c r="C39" t="s">
         <v>70</v>
@@ -1730,10 +1787,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
+        <v>141</v>
+      </c>
+      <c r="B40" t="s">
         <v>142</v>
-      </c>
-      <c r="B40" t="s">
-        <v>143</v>
       </c>
       <c r="C40" t="s">
         <v>70</v>
@@ -1741,10 +1798,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>143</v>
+      </c>
+      <c r="B41" t="s">
         <v>144</v>
-      </c>
-      <c r="B41" t="s">
-        <v>145</v>
       </c>
       <c r="C41" t="s">
         <v>70</v>
@@ -1752,10 +1809,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>145</v>
+      </c>
+      <c r="B42" t="s">
         <v>146</v>
-      </c>
-      <c r="B42" t="s">
-        <v>147</v>
       </c>
       <c r="C42" t="s">
         <v>70</v>
@@ -1763,10 +1820,10 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
+        <v>147</v>
+      </c>
+      <c r="B43" t="s">
         <v>148</v>
-      </c>
-      <c r="B43" t="s">
-        <v>149</v>
       </c>
       <c r="C43" t="s">
         <v>70</v>
@@ -1774,21 +1831,21 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
+        <v>149</v>
+      </c>
+      <c r="B44" t="s">
         <v>150</v>
       </c>
-      <c r="B44" t="s">
-        <v>151</v>
-      </c>
       <c r="C44" t="s">
-        <v>152</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B45" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C45" t="s">
         <v>70</v>
@@ -1796,21 +1853,21 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B46" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C46" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B47" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C47" t="s">
         <v>70</v>
@@ -1818,10 +1875,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B48" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C48" t="s">
         <v>70</v>
@@ -1829,10 +1886,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B49" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C49" t="s">
         <v>70</v>
@@ -1840,10 +1897,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B50" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C50" t="s">
         <v>70</v>
@@ -1851,21 +1908,21 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
+        <v>163</v>
+      </c>
+      <c r="B51" t="s">
+        <v>164</v>
+      </c>
+      <c r="C51" t="s">
         <v>165</v>
-      </c>
-      <c r="B51" t="s">
-        <v>166</v>
-      </c>
-      <c r="C51" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>166</v>
+      </c>
+      <c r="B52" t="s">
         <v>167</v>
-      </c>
-      <c r="B52" t="s">
-        <v>168</v>
       </c>
       <c r="C52" t="s">
         <v>70</v>
@@ -1873,10 +1930,10 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>168</v>
+      </c>
+      <c r="B53" t="s">
         <v>169</v>
-      </c>
-      <c r="B53" t="s">
-        <v>170</v>
       </c>
       <c r="C53" t="s">
         <v>70</v>
@@ -1884,21 +1941,21 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
+        <v>170</v>
+      </c>
+      <c r="B54" t="s">
         <v>171</v>
       </c>
-      <c r="B54" t="s">
-        <v>172</v>
-      </c>
       <c r="C54" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
+        <v>172</v>
+      </c>
+      <c r="B55" t="s">
         <v>173</v>
-      </c>
-      <c r="B55" t="s">
-        <v>98</v>
       </c>
       <c r="C55" t="s">
         <v>70</v>
@@ -1945,6 +2002,116 @@
         <v>181</v>
       </c>
       <c r="C59" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>182</v>
+      </c>
+      <c r="B60" t="s">
+        <v>183</v>
+      </c>
+      <c r="C60" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>184</v>
+      </c>
+      <c r="B61" t="s">
+        <v>185</v>
+      </c>
+      <c r="C61" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>186</v>
+      </c>
+      <c r="B62" t="s">
+        <v>187</v>
+      </c>
+      <c r="C62" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>188</v>
+      </c>
+      <c r="B63" t="s">
+        <v>98</v>
+      </c>
+      <c r="C63" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>189</v>
+      </c>
+      <c r="B64" t="s">
+        <v>190</v>
+      </c>
+      <c r="C64" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>191</v>
+      </c>
+      <c r="B65" t="s">
+        <v>192</v>
+      </c>
+      <c r="C65" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>193</v>
+      </c>
+      <c r="B66" t="s">
+        <v>194</v>
+      </c>
+      <c r="C66" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>195</v>
+      </c>
+      <c r="B67" t="s">
+        <v>196</v>
+      </c>
+      <c r="C67" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>197</v>
+      </c>
+      <c r="B68" t="s">
+        <v>198</v>
+      </c>
+      <c r="C68" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>199</v>
+      </c>
+      <c r="B69" t="s">
+        <v>200</v>
+      </c>
+      <c r="C69" t="s">
         <v>70</v>
       </c>
     </row>

</xml_diff>